<commit_message>
fix(7.2): a Total Row declared as Excel declares it, so example 2 opens
Excel wouldn't open copilot/examples/02_summary_and_total_row.xlsx without a repair, and
the repair dropped Table by_job. Its Total Row's cells were written, but the Table's
columns didn't declare them, and its filter reached into the Total Row. new_table now
declares each column as Excel does: a label, sum or max for a SUBTOTAL of the column
itself, or custom with the formula. The filter stops above the Total Row. contents
compares those declarations, and a new test reads every example and eval workbook the
way Excel reads a Table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/copilot/examples/02_summary_and_total_row.xlsx
+++ b/copilot/examples/02_summary_and_total_row.xlsx
@@ -193,13 +193,13 @@
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="by_job" displayName="by_job" ref="A1:E5" headerRowCount="1" totalsRowCount="1">
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:E4"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="job_id"/>
-    <tableColumn id="2" name="total_mins"/>
-    <tableColumn id="3" name="runs"/>
-    <tableColumn id="4" name="failed"/>
-    <tableColumn id="5" name="longest"/>
+    <tableColumn id="1" name="job_id" totalsRowLabel="Total"/>
+    <tableColumn id="2" name="total_mins" totalsRowFunction="sum"/>
+    <tableColumn id="3" name="runs" totalsRowFunction="sum"/>
+    <tableColumn id="4" name="failed" totalsRowFunction="sum"/>
+    <tableColumn id="5" name="longest" totalsRowFunction="max"/>
   </tableColumns>
 </table>
 </file>

</xml_diff>

<commit_message>
sqlglot Composer 7.2, exported 2026-10-29 18:12
Generated from dev 2a37a055416d8fbe39cfc34a4d19166a31caa338 by tools/export_clean.py. Never edit this branch by hand.
</commit_message>
<xml_diff>
--- a/copilot/examples/02_summary_and_total_row.xlsx
+++ b/copilot/examples/02_summary_and_total_row.xlsx
@@ -193,13 +193,13 @@
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="by_job" displayName="by_job" ref="A1:E5" headerRowCount="1" totalsRowCount="1">
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:E4"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="job_id"/>
-    <tableColumn id="2" name="total_mins"/>
-    <tableColumn id="3" name="runs"/>
-    <tableColumn id="4" name="failed"/>
-    <tableColumn id="5" name="longest"/>
+    <tableColumn id="1" name="job_id" totalsRowLabel="Total"/>
+    <tableColumn id="2" name="total_mins" totalsRowFunction="sum"/>
+    <tableColumn id="3" name="runs" totalsRowFunction="sum"/>
+    <tableColumn id="4" name="failed" totalsRowFunction="sum"/>
+    <tableColumn id="5" name="longest" totalsRowFunction="max"/>
   </tableColumns>
 </table>
 </file>

</xml_diff>